<commit_message>
Update requirement and implement terminal.
</commit_message>
<xml_diff>
--- a/Doc/Requirements.xlsx
+++ b/Doc/Requirements.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\D\Code\git\StockAnalysisSystem\Doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8924AFE-53E3-45F4-ABEC-B722D122B93C}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{908EB43D-625C-4427-BA9D-017408E2151F}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,17 +17,26 @@
     <sheet name="Product Requirement - WHAT" sheetId="2" r:id="rId2"/>
     <sheet name="Feature - HOW" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="965" uniqueCount="583">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="984" uniqueCount="602">
   <si>
     <t>ID</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -774,9 +783,6 @@
     <t>没有企业号，无法测试</t>
   </si>
   <si>
-    <t>终端服务</t>
-  </si>
-  <si>
     <t>用户可通过某种终端进行交互</t>
   </si>
   <si>
@@ -1922,6 +1928,86 @@
   </si>
   <si>
     <t>盯盘服务</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>终端服务</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>终端服务</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>获取分析结果</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>观察</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>通用规则</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>股票代码不需要加上后缀</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>需要输入股票代码的地方可以直接输入股票名</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>作用：直接返回简略的分析结果和评分；同时给出完整分析结果的链接</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>格式：“分析结果” + 股票代码；“分析结果”可以出现在股票代码或股票名的前面或后面</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">           输入股票代码或股票名，如果正确且唯一，默认返回分析结果</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>格式：“观察” + 股票代码</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>交互命令</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>作用：将该股票加入观察列表，并将当前的价格作为基准</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>设置基准价格</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>格式：“设置基准” + 股票代码 + 价格</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>i</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>作用：为股票设置观察的价格基准；如果该股票没有加入观察列表，则自动加入观察列表；如果没有价格参数，则使用当前价格</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>“+”号分隔的部分实际应以空格分隔</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>设置通知价格</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>推送</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -3505,7 +3591,7 @@
     </row>
     <row r="52" spans="4:8" outlineLevel="3" x14ac:dyDescent="0.25">
       <c r="F52" s="1" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="G52" s="4" t="s">
         <v>214</v>
@@ -3513,7 +3599,7 @@
     </row>
     <row r="53" spans="4:8" outlineLevel="3" x14ac:dyDescent="0.25">
       <c r="F53" s="1" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="G53" s="4" t="s">
         <v>215</v>
@@ -3527,12 +3613,12 @@
         <v>210</v>
       </c>
       <c r="H54" s="2" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
     </row>
     <row r="55" spans="4:8" outlineLevel="3" x14ac:dyDescent="0.25">
       <c r="F55" s="1" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="G55" s="4" t="s">
         <v>215</v>
@@ -3589,7 +3675,7 @@
     </row>
     <row r="62" spans="4:8" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="E62" s="1" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="G62" s="4" t="s">
         <v>215</v>
@@ -3597,7 +3683,7 @@
     </row>
     <row r="63" spans="4:8" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="E63" s="1" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="G63" s="4" t="s">
         <v>215</v>
@@ -3618,13 +3704,13 @@
     </row>
     <row r="66" spans="4:7" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="E66" s="1" t="s">
+        <v>259</v>
+      </c>
+      <c r="F66" s="1" t="s">
         <v>260</v>
       </c>
-      <c r="F66" s="1" t="s">
+      <c r="G66" s="4" t="s">
         <v>261</v>
-      </c>
-      <c r="G66" s="4" t="s">
-        <v>262</v>
       </c>
     </row>
     <row r="67" spans="4:7" outlineLevel="2" x14ac:dyDescent="0.25">
@@ -3885,7 +3971,7 @@
     </row>
     <row r="117" spans="4:6" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="E117" s="1" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="118" spans="4:6" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -3895,71 +3981,71 @@
     </row>
     <row r="119" spans="4:6" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="E119" s="1" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="120" spans="4:6" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="F120" s="1" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="121" spans="4:6" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="F121" s="1" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="122" spans="4:6" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="E122" s="1" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
     </row>
     <row r="123" spans="4:6" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="F123" s="1" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
     </row>
     <row r="124" spans="4:6" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="F124" s="1" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
     </row>
     <row r="125" spans="4:6" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="F125" s="1" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
     </row>
     <row r="126" spans="4:6" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="E126" s="1" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
     </row>
     <row r="127" spans="4:6" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="E127" s="1" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="F127" s="1" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
     </row>
     <row r="128" spans="4:6" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="E128" s="1" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="F128" s="1" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
     </row>
     <row r="129" spans="1:7" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="E129" s="1" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="F129" s="1" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="130" spans="1:7" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="E130" s="1" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
     </row>
     <row r="131" spans="1:7" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -3969,53 +4055,53 @@
     </row>
     <row r="132" spans="1:7" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="E132" s="1" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
     </row>
     <row r="133" spans="1:7" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="E133" s="1" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="134" spans="1:7" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="D134" s="1" t="s">
-        <v>221</v>
+        <v>582</v>
       </c>
       <c r="F134" s="1" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="G134" s="4"/>
     </row>
     <row r="135" spans="1:7" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="E135" s="1" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="F135" s="1" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="G135" s="4"/>
     </row>
     <row r="136" spans="1:7" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="E136" s="1" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="F136" s="1" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="G136" s="4"/>
     </row>
     <row r="137" spans="1:7" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="A137" s="1" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="E137" s="1" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="G137" s="4"/>
     </row>
     <row r="138" spans="1:7" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="E138" s="1" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="G138" s="4"/>
     </row>
@@ -4027,25 +4113,25 @@
     </row>
     <row r="140" spans="1:7" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="F140" s="1" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="G140" s="4"/>
     </row>
     <row r="141" spans="1:7" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="A141" s="1" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="F141" s="1" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="G141" s="4"/>
     </row>
     <row r="142" spans="1:7" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="A142" s="1" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="F142" s="1" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="G142" s="4"/>
     </row>
@@ -4057,13 +4143,13 @@
     </row>
     <row r="144" spans="1:7" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="F144" s="1" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="G144" s="4"/>
     </row>
     <row r="145" spans="1:7" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="F145" s="1" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="G145" s="4"/>
     </row>
@@ -4075,7 +4161,7 @@
     </row>
     <row r="147" spans="1:7" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A147" s="1" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="D147" s="1" t="s">
         <v>189</v>
@@ -4084,13 +4170,13 @@
     </row>
     <row r="148" spans="1:7" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="E148" s="1" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G148" s="4"/>
     </row>
     <row r="149" spans="1:7" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="E149" s="1" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="G149" s="4"/>
     </row>
@@ -4102,13 +4188,13 @@
     </row>
     <row r="151" spans="1:7" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="E151" s="1" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G151" s="4"/>
     </row>
     <row r="152" spans="1:7" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="E152" s="1" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="G152" s="4"/>
     </row>
@@ -4136,7 +4222,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:L232"/>
+  <dimension ref="A1:L266"/>
   <sheetFormatPr defaultRowHeight="13.8" outlineLevelRow="2" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="16.6640625" bestFit="1" customWidth="1"/>
@@ -4179,7 +4265,7 @@
       <c r="B4" s="1"/>
       <c r="C4" s="2"/>
       <c r="D4" s="1" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
     </row>
     <row r="5" spans="1:7" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -4188,7 +4274,7 @@
       <c r="C5" s="2"/>
       <c r="D5" s="1"/>
       <c r="E5" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
     </row>
     <row r="6" spans="1:7" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -4197,7 +4283,7 @@
       <c r="C6" s="2"/>
       <c r="D6" s="1"/>
       <c r="E6" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="7" spans="1:7" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -4206,7 +4292,7 @@
       <c r="C7" s="2"/>
       <c r="D7" s="1"/>
       <c r="F7" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
     </row>
     <row r="8" spans="1:7" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -4215,10 +4301,10 @@
       <c r="C8" s="2"/>
       <c r="D8" s="1"/>
       <c r="F8" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="G8" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
     </row>
     <row r="9" spans="1:7" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -4227,10 +4313,10 @@
       <c r="C9" s="2"/>
       <c r="D9" s="1"/>
       <c r="F9" t="s">
+        <v>383</v>
+      </c>
+      <c r="G9" t="s">
         <v>384</v>
-      </c>
-      <c r="G9" t="s">
-        <v>385</v>
       </c>
     </row>
     <row r="10" spans="1:7" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -4239,10 +4325,10 @@
       <c r="C10" s="2"/>
       <c r="D10" s="1"/>
       <c r="F10" t="s">
+        <v>385</v>
+      </c>
+      <c r="G10" t="s">
         <v>386</v>
-      </c>
-      <c r="G10" t="s">
-        <v>387</v>
       </c>
     </row>
     <row r="11" spans="1:7" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -4251,7 +4337,7 @@
       <c r="C11" s="2"/>
       <c r="D11" s="1"/>
       <c r="E11" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
     </row>
     <row r="12" spans="1:7" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -4260,7 +4346,7 @@
       <c r="C12" s="2"/>
       <c r="D12" s="1"/>
       <c r="F12" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
     </row>
     <row r="13" spans="1:7" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -4269,10 +4355,10 @@
       <c r="C13" s="2"/>
       <c r="D13" s="1"/>
       <c r="F13" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="G13" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
     </row>
     <row r="14" spans="1:7" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -4281,7 +4367,7 @@
       <c r="C14" s="2"/>
       <c r="D14" s="1"/>
       <c r="E14" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
     </row>
     <row r="15" spans="1:7" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -4290,7 +4376,7 @@
       <c r="C15" s="2"/>
       <c r="D15" s="1"/>
       <c r="F15" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
     </row>
     <row r="16" spans="1:7" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -4299,7 +4385,7 @@
       <c r="C16" s="2"/>
       <c r="D16" s="1"/>
       <c r="F16" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
     </row>
     <row r="17" spans="1:7" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -4307,7 +4393,7 @@
       <c r="B17" s="1"/>
       <c r="C17" s="2"/>
       <c r="D17" s="1" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
@@ -4315,7 +4401,7 @@
       <c r="B18" s="1"/>
       <c r="C18" s="1"/>
       <c r="D18" s="1" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
     </row>
     <row r="19" spans="1:7" outlineLevel="1" collapsed="1" x14ac:dyDescent="0.25">
@@ -4324,7 +4410,7 @@
       <c r="C19" s="1"/>
       <c r="D19" s="1"/>
       <c r="E19" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="20" spans="1:7" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
@@ -4333,10 +4419,10 @@
       <c r="C20" s="1"/>
       <c r="D20" s="1"/>
       <c r="F20" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="G20" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
     </row>
     <row r="21" spans="1:7" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
@@ -4345,7 +4431,7 @@
       <c r="C21" s="1"/>
       <c r="D21" s="1"/>
       <c r="F21" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
     </row>
     <row r="22" spans="1:7" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
@@ -4360,7 +4446,7 @@
       <c r="C23" s="1"/>
       <c r="D23" s="1"/>
       <c r="F23" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
     </row>
     <row r="24" spans="1:7" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
@@ -4369,7 +4455,7 @@
       <c r="C24" s="1"/>
       <c r="D24" s="1"/>
       <c r="G24" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
     </row>
     <row r="25" spans="1:7" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
@@ -4378,7 +4464,7 @@
       <c r="C25" s="1"/>
       <c r="D25" s="1"/>
       <c r="G25" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
     </row>
     <row r="26" spans="1:7" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
@@ -4387,7 +4473,7 @@
       <c r="C26" s="1"/>
       <c r="D26" s="1"/>
       <c r="G26" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
     </row>
     <row r="27" spans="1:7" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
@@ -4402,7 +4488,7 @@
       <c r="C28" s="1"/>
       <c r="D28" s="1"/>
       <c r="F28" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
     </row>
     <row r="29" spans="1:7" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
@@ -4411,7 +4497,7 @@
       <c r="C29" s="1"/>
       <c r="D29" s="1"/>
       <c r="G29" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
     </row>
     <row r="30" spans="1:7" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
@@ -4420,7 +4506,7 @@
       <c r="C30" s="1"/>
       <c r="D30" s="1"/>
       <c r="G30" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
     </row>
     <row r="31" spans="1:7" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
@@ -4429,7 +4515,7 @@
       <c r="C31" s="1"/>
       <c r="D31" s="1"/>
       <c r="G31" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
     </row>
     <row r="32" spans="1:7" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
@@ -4438,7 +4524,7 @@
       <c r="C32" s="1"/>
       <c r="D32" s="1"/>
       <c r="F32" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
     </row>
     <row r="33" spans="1:12" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
@@ -4447,7 +4533,7 @@
       <c r="C33" s="1"/>
       <c r="D33" s="1"/>
       <c r="G33" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="34" spans="1:12" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
@@ -4456,7 +4542,7 @@
       <c r="C34" s="1"/>
       <c r="D34" s="1"/>
       <c r="G34" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
     </row>
     <row r="35" spans="1:12" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
@@ -4465,7 +4551,7 @@
       <c r="C35" s="1"/>
       <c r="D35" s="1"/>
       <c r="G35" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
     </row>
     <row r="36" spans="1:12" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
@@ -4474,58 +4560,58 @@
       <c r="C36" s="1"/>
       <c r="D36" s="1"/>
       <c r="E36" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
     </row>
     <row r="37" spans="1:12" outlineLevel="1" collapsed="1" x14ac:dyDescent="0.25">
       <c r="E37" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="38" spans="1:12" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="F38" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
     </row>
     <row r="39" spans="1:12" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25"/>
     <row r="40" spans="1:12" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="F40" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="G40" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="H40" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="I40" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="J40" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="K40" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="L40" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
     </row>
     <row r="41" spans="1:12" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="F41" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="G41" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="H41" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="I41" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="J41" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="L41" t="s">
         <v>214</v>
@@ -4533,19 +4619,19 @@
     </row>
     <row r="42" spans="1:12" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="F42" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="G42" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="H42" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="I42" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="J42" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="L42" t="s">
         <v>214</v>
@@ -4553,19 +4639,19 @@
     </row>
     <row r="43" spans="1:12" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="F43" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="G43" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="H43" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="I43" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="J43" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="L43" t="s">
         <v>214</v>
@@ -4573,19 +4659,19 @@
     </row>
     <row r="44" spans="1:12" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="F44" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="G44" t="s">
+        <v>276</v>
+      </c>
+      <c r="H44" t="s">
+        <v>310</v>
+      </c>
+      <c r="I44" t="s">
         <v>277</v>
       </c>
-      <c r="H44" t="s">
-        <v>311</v>
-      </c>
-      <c r="I44" t="s">
-        <v>278</v>
-      </c>
       <c r="J44" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="L44" t="s">
         <v>215</v>
@@ -4593,19 +4679,19 @@
     </row>
     <row r="45" spans="1:12" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="F45" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="G45" t="s">
+        <v>279</v>
+      </c>
+      <c r="H45" t="s">
+        <v>310</v>
+      </c>
+      <c r="I45" t="s">
         <v>280</v>
       </c>
-      <c r="H45" t="s">
-        <v>311</v>
-      </c>
-      <c r="I45" t="s">
-        <v>281</v>
-      </c>
       <c r="J45" t="s">
-        <v>540</v>
+        <v>539</v>
       </c>
       <c r="L45" t="s">
         <v>215</v>
@@ -4613,19 +4699,19 @@
     </row>
     <row r="46" spans="1:12" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="F46" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="G46" t="s">
+        <v>281</v>
+      </c>
+      <c r="H46" t="s">
+        <v>310</v>
+      </c>
+      <c r="I46" t="s">
         <v>282</v>
       </c>
-      <c r="H46" t="s">
-        <v>311</v>
-      </c>
-      <c r="I46" t="s">
-        <v>283</v>
-      </c>
       <c r="J46" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="L46" t="s">
         <v>214</v>
@@ -4633,16 +4719,16 @@
     </row>
     <row r="47" spans="1:12" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="F47" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="G47" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="H47" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="I47" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="L47" t="s">
         <v>214</v>
@@ -4650,19 +4736,19 @@
     </row>
     <row r="48" spans="1:12" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="F48" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G48" t="s">
+        <v>284</v>
+      </c>
+      <c r="H48" t="s">
+        <v>310</v>
+      </c>
+      <c r="I48" t="s">
         <v>285</v>
       </c>
-      <c r="H48" t="s">
-        <v>311</v>
-      </c>
-      <c r="I48" t="s">
-        <v>286</v>
-      </c>
       <c r="J48" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="L48" t="s">
         <v>214</v>
@@ -4670,19 +4756,19 @@
     </row>
     <row r="49" spans="6:12" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="F49" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="G49" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="H49" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="I49" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="J49" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="L49" t="s">
         <v>214</v>
@@ -4690,19 +4776,19 @@
     </row>
     <row r="50" spans="6:12" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="F50" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="G50" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="H50" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="I50" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="J50" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="L50" t="s">
         <v>214</v>
@@ -4710,19 +4796,19 @@
     </row>
     <row r="51" spans="6:12" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="F51" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="G51" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="H51" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="I51" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="J51" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="L51" t="s">
         <v>214</v>
@@ -4730,19 +4816,19 @@
     </row>
     <row r="52" spans="6:12" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="F52" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="G52" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="H52" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="I52" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="J52" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="L52" t="s">
         <v>214</v>
@@ -4750,19 +4836,19 @@
     </row>
     <row r="53" spans="6:12" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="F53" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="G53" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="H53" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="I53" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="J53" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="L53" t="s">
         <v>214</v>
@@ -4770,16 +4856,16 @@
     </row>
     <row r="54" spans="6:12" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="F54" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="G54" t="s">
+        <v>293</v>
+      </c>
+      <c r="H54" t="s">
+        <v>310</v>
+      </c>
+      <c r="I54" t="s">
         <v>294</v>
-      </c>
-      <c r="H54" t="s">
-        <v>311</v>
-      </c>
-      <c r="I54" t="s">
-        <v>295</v>
       </c>
       <c r="L54" t="s">
         <v>214</v>
@@ -4787,16 +4873,16 @@
     </row>
     <row r="55" spans="6:12" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="F55" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="G55" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="H55" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="I55" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="L55" t="s">
         <v>214</v>
@@ -4804,16 +4890,16 @@
     </row>
     <row r="56" spans="6:12" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="F56" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="G56" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="H56" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="I56" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="L56" t="s">
         <v>214</v>
@@ -4821,19 +4907,19 @@
     </row>
     <row r="57" spans="6:12" ht="27.6" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="F57" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="G57" t="s">
+        <v>298</v>
+      </c>
+      <c r="H57" t="s">
+        <v>311</v>
+      </c>
+      <c r="I57" t="s">
         <v>299</v>
       </c>
-      <c r="H57" t="s">
-        <v>312</v>
-      </c>
-      <c r="I57" t="s">
-        <v>300</v>
-      </c>
       <c r="K57" s="7" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="L57" t="s">
         <v>214</v>
@@ -4841,19 +4927,19 @@
     </row>
     <row r="58" spans="6:12" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="F58" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="G58" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="H58" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="I58" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="J58" t="s">
-        <v>538</v>
+        <v>537</v>
       </c>
       <c r="L58" t="s">
         <v>214</v>
@@ -4861,19 +4947,19 @@
     </row>
     <row r="59" spans="6:12" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="F59" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="G59" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="H59" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="I59" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="J59" t="s">
-        <v>538</v>
+        <v>537</v>
       </c>
       <c r="L59" t="s">
         <v>214</v>
@@ -4881,19 +4967,19 @@
     </row>
     <row r="60" spans="6:12" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="F60" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="G60" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="H60" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="I60" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="J60" t="s">
-        <v>538</v>
+        <v>537</v>
       </c>
       <c r="L60" t="s">
         <v>214</v>
@@ -4901,16 +4987,16 @@
     </row>
     <row r="61" spans="6:12" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="F61" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="G61" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="H61" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="I61" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="L61" t="s">
         <v>214</v>
@@ -4918,16 +5004,16 @@
     </row>
     <row r="62" spans="6:12" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="F62" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="G62" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="H62" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="I62" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="L62" t="s">
         <v>214</v>
@@ -4935,16 +5021,16 @@
     </row>
     <row r="63" spans="6:12" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="F63" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="G63" t="s">
+        <v>305</v>
+      </c>
+      <c r="H63" t="s">
+        <v>310</v>
+      </c>
+      <c r="I63" t="s">
         <v>306</v>
-      </c>
-      <c r="H63" t="s">
-        <v>311</v>
-      </c>
-      <c r="I63" t="s">
-        <v>307</v>
       </c>
       <c r="L63" t="s">
         <v>214</v>
@@ -4953,245 +5039,245 @@
     <row r="64" spans="6:12" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25"/>
     <row r="65" spans="5:12" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="F65" t="s">
-        <v>536</v>
+        <v>535</v>
       </c>
       <c r="G65" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="H65" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="I65" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="J65" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="L65" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
     </row>
     <row r="66" spans="5:12" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="F66" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="G66" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H66" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="I66" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="J66" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="L66" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
     </row>
     <row r="67" spans="5:12" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="F67" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="G67" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="H67" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="I67" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="J67" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="L67" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
     </row>
     <row r="68" spans="5:12" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="F68" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="G68" t="s">
-        <v>528</v>
+        <v>527</v>
       </c>
       <c r="H68" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="I68" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="L68" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
     </row>
     <row r="69" spans="5:12" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25"/>
     <row r="70" spans="5:12" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="F70" t="s">
-        <v>545</v>
+        <v>544</v>
       </c>
       <c r="G70" t="s">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="H70" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="I70" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="J70" t="s">
-        <v>538</v>
+        <v>537</v>
       </c>
       <c r="L70" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
     </row>
     <row r="71" spans="5:12" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="F71" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="G71" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="H71" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="I71" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="J71" t="s">
-        <v>538</v>
+        <v>537</v>
       </c>
       <c r="L71" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
     </row>
     <row r="72" spans="5:12" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="F72" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="G72" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="H72" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="I72" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="J72" t="s">
-        <v>537</v>
+        <v>536</v>
       </c>
       <c r="L72" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
     </row>
     <row r="73" spans="5:12" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="F73" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
       <c r="G73" t="s">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="H73" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="I73" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="J73" t="s">
-        <v>537</v>
+        <v>536</v>
       </c>
       <c r="L73" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
     </row>
     <row r="74" spans="5:12" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="F74" t="s">
+        <v>548</v>
+      </c>
+      <c r="G74" t="s">
         <v>549</v>
       </c>
-      <c r="G74" t="s">
-        <v>550</v>
-      </c>
       <c r="H74" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="I74" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="J74" t="s">
-        <v>537</v>
+        <v>536</v>
       </c>
       <c r="L74" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
     </row>
     <row r="75" spans="5:12" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="F75" t="s">
+        <v>550</v>
+      </c>
+      <c r="G75" t="s">
         <v>551</v>
       </c>
-      <c r="G75" t="s">
+      <c r="H75" t="s">
+        <v>310</v>
+      </c>
+      <c r="I75" t="s">
         <v>552</v>
       </c>
-      <c r="H75" t="s">
-        <v>311</v>
-      </c>
-      <c r="I75" t="s">
-        <v>553</v>
-      </c>
       <c r="J75" t="s">
-        <v>537</v>
+        <v>536</v>
       </c>
       <c r="L75" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
     </row>
     <row r="76" spans="5:12" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25"/>
     <row r="77" spans="5:12" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="E77" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
     </row>
     <row r="78" spans="5:12" outlineLevel="1" collapsed="1" x14ac:dyDescent="0.25">
       <c r="E78" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
     </row>
     <row r="79" spans="5:12" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="F79" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
     </row>
     <row r="80" spans="5:12" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25"/>
     <row r="81" spans="7:11" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="G81" t="s">
+        <v>265</v>
+      </c>
+      <c r="H81" t="s">
         <v>266</v>
       </c>
-      <c r="H81" t="s">
-        <v>267</v>
-      </c>
       <c r="I81" t="s">
+        <v>337</v>
+      </c>
+      <c r="J81" t="s">
         <v>338</v>
       </c>
-      <c r="J81" t="s">
-        <v>339</v>
-      </c>
       <c r="K81" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
     </row>
     <row r="82" spans="7:11" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="G82" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="H82" t="s">
+        <v>263</v>
+      </c>
+      <c r="I82" s="5" t="s">
         <v>264</v>
-      </c>
-      <c r="I82" s="5" t="s">
-        <v>265</v>
       </c>
       <c r="K82" t="s">
         <v>214</v>
@@ -5199,13 +5285,13 @@
     </row>
     <row r="83" spans="7:11" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="G83" t="s">
+        <v>269</v>
+      </c>
+      <c r="H83" t="s">
         <v>270</v>
       </c>
-      <c r="H83" t="s">
-        <v>271</v>
-      </c>
       <c r="I83" s="5" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="K83" t="s">
         <v>214</v>
@@ -5213,13 +5299,13 @@
     </row>
     <row r="84" spans="7:11" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="G84" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="H84" t="s">
+        <v>339</v>
+      </c>
+      <c r="I84" s="5" t="s">
         <v>340</v>
-      </c>
-      <c r="I84" s="5" t="s">
-        <v>341</v>
       </c>
       <c r="K84" t="s">
         <v>214</v>
@@ -5227,13 +5313,13 @@
     </row>
     <row r="85" spans="7:11" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="G85" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="H85" t="s">
+        <v>341</v>
+      </c>
+      <c r="I85" s="5" t="s">
         <v>342</v>
-      </c>
-      <c r="I85" s="5" t="s">
-        <v>343</v>
       </c>
       <c r="K85" t="s">
         <v>214</v>
@@ -5241,13 +5327,13 @@
     </row>
     <row r="86" spans="7:11" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="G86" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="H86" t="s">
+        <v>360</v>
+      </c>
+      <c r="I86" s="5" t="s">
         <v>361</v>
-      </c>
-      <c r="I86" s="5" t="s">
-        <v>362</v>
       </c>
       <c r="K86" t="s">
         <v>214</v>
@@ -5255,13 +5341,13 @@
     </row>
     <row r="87" spans="7:11" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="G87" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="H87" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="I87" s="5" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="K87" t="s">
         <v>214</v>
@@ -5269,13 +5355,13 @@
     </row>
     <row r="88" spans="7:11" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="G88" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="H88" t="s">
+        <v>347</v>
+      </c>
+      <c r="I88" s="5" t="s">
         <v>348</v>
-      </c>
-      <c r="I88" s="5" t="s">
-        <v>349</v>
       </c>
       <c r="K88" t="s">
         <v>214</v>
@@ -5283,13 +5369,13 @@
     </row>
     <row r="89" spans="7:11" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="G89" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="H89" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="I89" s="5" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="K89" t="s">
         <v>214</v>
@@ -5297,13 +5383,13 @@
     </row>
     <row r="90" spans="7:11" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="G90" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="H90" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="I90" s="5" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="K90" t="s">
         <v>214</v>
@@ -5311,13 +5397,13 @@
     </row>
     <row r="91" spans="7:11" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="G91" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="H91" t="s">
+        <v>352</v>
+      </c>
+      <c r="I91" s="5" t="s">
         <v>353</v>
-      </c>
-      <c r="I91" s="5" t="s">
-        <v>354</v>
       </c>
       <c r="K91" t="s">
         <v>214</v>
@@ -5325,13 +5411,13 @@
     </row>
     <row r="92" spans="7:11" ht="41.4" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="G92" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="H92" s="7" t="s">
+        <v>358</v>
+      </c>
+      <c r="I92" s="6" t="s">
         <v>359</v>
-      </c>
-      <c r="I92" s="6" t="s">
-        <v>360</v>
       </c>
       <c r="K92" t="s">
         <v>214</v>
@@ -5339,13 +5425,13 @@
     </row>
     <row r="93" spans="7:11" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="G93" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="H93" t="s">
+        <v>362</v>
+      </c>
+      <c r="I93" s="5" t="s">
         <v>363</v>
-      </c>
-      <c r="I93" s="5" t="s">
-        <v>364</v>
       </c>
       <c r="K93" t="s">
         <v>214</v>
@@ -5353,13 +5439,13 @@
     </row>
     <row r="94" spans="7:11" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="G94" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="H94" t="s">
+        <v>364</v>
+      </c>
+      <c r="I94" s="5" t="s">
         <v>365</v>
-      </c>
-      <c r="I94" s="5" t="s">
-        <v>366</v>
       </c>
       <c r="K94" t="s">
         <v>214</v>
@@ -5367,13 +5453,13 @@
     </row>
     <row r="95" spans="7:11" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="G95" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="H95" t="s">
+        <v>366</v>
+      </c>
+      <c r="I95" s="5" t="s">
         <v>367</v>
-      </c>
-      <c r="I95" s="5" t="s">
-        <v>368</v>
       </c>
       <c r="K95" t="s">
         <v>214</v>
@@ -5381,13 +5467,13 @@
     </row>
     <row r="96" spans="7:11" ht="27.6" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="G96" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="H96" s="7" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="I96" s="6" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="K96" t="s">
         <v>214</v>
@@ -5395,13 +5481,13 @@
     </row>
     <row r="97" spans="7:11" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="G97" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="H97" t="s">
+        <v>368</v>
+      </c>
+      <c r="I97" s="5" t="s">
         <v>369</v>
-      </c>
-      <c r="I97" s="5" t="s">
-        <v>370</v>
       </c>
       <c r="K97" t="s">
         <v>214</v>
@@ -5409,13 +5495,13 @@
     </row>
     <row r="98" spans="7:11" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="G98" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="H98" t="s">
+        <v>370</v>
+      </c>
+      <c r="I98" s="5" t="s">
         <v>371</v>
-      </c>
-      <c r="I98" s="5" t="s">
-        <v>372</v>
       </c>
       <c r="K98" t="s">
         <v>214</v>
@@ -5423,13 +5509,13 @@
     </row>
     <row r="99" spans="7:11" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="G99" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="H99" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="I99" s="5" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="K99" t="s">
         <v>214</v>
@@ -5437,13 +5523,13 @@
     </row>
     <row r="100" spans="7:11" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="G100" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="H100" t="s">
+        <v>373</v>
+      </c>
+      <c r="I100" s="5" t="s">
         <v>374</v>
-      </c>
-      <c r="I100" s="5" t="s">
-        <v>375</v>
       </c>
       <c r="K100" t="s">
         <v>214</v>
@@ -5454,58 +5540,58 @@
     </row>
     <row r="102" spans="7:11" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="G102" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="H102" t="s">
+        <v>565</v>
+      </c>
+      <c r="I102" s="5" t="s">
         <v>566</v>
       </c>
-      <c r="I102" s="5" t="s">
-        <v>567</v>
-      </c>
       <c r="K102" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
     </row>
     <row r="103" spans="7:11" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="G103" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H103" t="s">
+        <v>567</v>
+      </c>
+      <c r="I103" s="5" t="s">
         <v>568</v>
       </c>
-      <c r="I103" s="5" t="s">
-        <v>569</v>
-      </c>
       <c r="K103" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
     </row>
     <row r="104" spans="7:11" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="G104" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="H104" t="s">
+        <v>569</v>
+      </c>
+      <c r="I104" s="5" t="s">
         <v>570</v>
       </c>
-      <c r="I104" s="5" t="s">
-        <v>571</v>
-      </c>
       <c r="K104" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
     </row>
     <row r="105" spans="7:11" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="G105" t="s">
-        <v>528</v>
+        <v>527</v>
       </c>
       <c r="H105" t="s">
+        <v>571</v>
+      </c>
+      <c r="I105" s="5" t="s">
         <v>572</v>
       </c>
-      <c r="I105" s="5" t="s">
+      <c r="K105" t="s">
         <v>573</v>
-      </c>
-      <c r="K105" t="s">
-        <v>574</v>
       </c>
     </row>
     <row r="106" spans="7:11" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
@@ -5513,86 +5599,86 @@
     </row>
     <row r="107" spans="7:11" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="G107" t="s">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="H107" t="s">
+        <v>553</v>
+      </c>
+      <c r="I107" s="5" t="s">
         <v>554</v>
       </c>
-      <c r="I107" s="5" t="s">
-        <v>555</v>
-      </c>
       <c r="K107" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
     </row>
     <row r="108" spans="7:11" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="G108" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="H108" t="s">
+        <v>555</v>
+      </c>
+      <c r="I108" s="5" t="s">
         <v>556</v>
       </c>
-      <c r="I108" s="5" t="s">
-        <v>557</v>
-      </c>
       <c r="K108" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
     </row>
     <row r="109" spans="7:11" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="G109" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="H109" t="s">
+        <v>557</v>
+      </c>
+      <c r="I109" s="5" t="s">
         <v>558</v>
       </c>
-      <c r="I109" s="5" t="s">
-        <v>559</v>
-      </c>
       <c r="K109" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
     </row>
     <row r="110" spans="7:11" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="G110" t="s">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="H110" t="s">
+        <v>559</v>
+      </c>
+      <c r="I110" s="5" t="s">
         <v>560</v>
       </c>
-      <c r="I110" s="5" t="s">
-        <v>561</v>
-      </c>
       <c r="K110" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
     </row>
     <row r="111" spans="7:11" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="G111" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="H111" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
       <c r="I111" s="5" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
       <c r="K111" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
     </row>
     <row r="112" spans="7:11" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="G112" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
       <c r="H112" t="s">
+        <v>563</v>
+      </c>
+      <c r="I112" s="5" t="s">
         <v>564</v>
       </c>
-      <c r="I112" s="5" t="s">
-        <v>565</v>
-      </c>
       <c r="K112" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
     </row>
     <row r="113" spans="4:11" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
@@ -5600,50 +5686,50 @@
     </row>
     <row r="114" spans="4:11" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="F114" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="I114" s="5"/>
       <c r="K114" s="8" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
     </row>
     <row r="115" spans="4:11" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="E115" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
     </row>
     <row r="116" spans="4:11" outlineLevel="1" collapsed="1" x14ac:dyDescent="0.25">
       <c r="E116" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
     </row>
     <row r="117" spans="4:11" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="E117" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
     </row>
     <row r="118" spans="4:11" outlineLevel="1" collapsed="1" x14ac:dyDescent="0.25">
       <c r="E118" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
     </row>
     <row r="119" spans="4:11" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="G119" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="H119" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="K119" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
     </row>
     <row r="120" spans="4:11" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="G120" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="H120" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="K120" t="s">
         <v>215</v>
@@ -5651,13 +5737,13 @@
     </row>
     <row r="121" spans="4:11" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="E121" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="G121" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="H121" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="K121" t="s">
         <v>215</v>
@@ -5666,131 +5752,131 @@
     <row r="122" spans="4:11" outlineLevel="1" x14ac:dyDescent="0.25"/>
     <row r="123" spans="4:11" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="D123" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
     </row>
     <row r="124" spans="4:11" x14ac:dyDescent="0.25">
       <c r="D124" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
     </row>
     <row r="125" spans="4:11" outlineLevel="1" collapsed="1" x14ac:dyDescent="0.25">
       <c r="E125" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="126" spans="4:11" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="F126" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="G126" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="127" spans="4:11" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="F127" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
     </row>
     <row r="128" spans="4:11" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25"/>
     <row r="129" spans="5:9" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="F129" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
     </row>
     <row r="130" spans="5:9" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="G130" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
     </row>
     <row r="131" spans="5:9" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="G131" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
     </row>
     <row r="132" spans="5:9" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="G132" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="H132" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
     </row>
     <row r="133" spans="5:9" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="G133" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="H133" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
     </row>
     <row r="134" spans="5:9" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="G134" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="H134" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
     </row>
     <row r="135" spans="5:9" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="G135" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="H135" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
     </row>
     <row r="136" spans="5:9" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="G136" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="H136" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
     </row>
     <row r="137" spans="5:9" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="G137" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="H137" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
     </row>
     <row r="138" spans="5:9" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="G138" t="s">
+        <v>432</v>
+      </c>
+      <c r="H138" t="s">
         <v>433</v>
-      </c>
-      <c r="H138" t="s">
-        <v>434</v>
       </c>
     </row>
     <row r="139" spans="5:9" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="G139" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
     </row>
     <row r="140" spans="5:9" outlineLevel="1" collapsed="1" x14ac:dyDescent="0.25">
       <c r="E140" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
     </row>
     <row r="141" spans="5:9" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="F141" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="H141" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="I141" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
     </row>
     <row r="142" spans="5:9" ht="55.2" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="F142" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="H142" s="7" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="I142" t="s">
         <v>214</v>
@@ -5798,10 +5884,10 @@
     </row>
     <row r="143" spans="5:9" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="F143" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="H143" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="I143" t="s">
         <v>214</v>
@@ -5809,7 +5895,7 @@
     </row>
     <row r="144" spans="5:9" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="F144" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="I144" t="s">
         <v>214</v>
@@ -5817,10 +5903,10 @@
     </row>
     <row r="145" spans="6:9" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="F145" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="H145" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="I145" t="s">
         <v>214</v>
@@ -5828,10 +5914,10 @@
     </row>
     <row r="146" spans="6:9" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="F146" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="H146" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="I146" t="s">
         <v>214</v>
@@ -5839,10 +5925,10 @@
     </row>
     <row r="147" spans="6:9" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="F147" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="H147" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="I147" t="s">
         <v>214</v>
@@ -5850,7 +5936,7 @@
     </row>
     <row r="148" spans="6:9" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="F148" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="I148" t="s">
         <v>214</v>
@@ -5858,7 +5944,7 @@
     </row>
     <row r="149" spans="6:9" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="F149" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="I149" t="s">
         <v>214</v>
@@ -5866,7 +5952,7 @@
     </row>
     <row r="150" spans="6:9" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="F150" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="I150" t="s">
         <v>214</v>
@@ -5874,7 +5960,7 @@
     </row>
     <row r="151" spans="6:9" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="F151" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="I151" t="s">
         <v>214</v>
@@ -5882,7 +5968,7 @@
     </row>
     <row r="152" spans="6:9" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="F152" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="I152" t="s">
         <v>214</v>
@@ -5890,7 +5976,7 @@
     </row>
     <row r="153" spans="6:9" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="F153" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="I153" t="s">
         <v>214</v>
@@ -5898,7 +5984,7 @@
     </row>
     <row r="154" spans="6:9" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="F154" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="I154" t="s">
         <v>214</v>
@@ -5906,7 +5992,7 @@
     </row>
     <row r="155" spans="6:9" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="F155" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="I155" t="s">
         <v>214</v>
@@ -5914,7 +6000,7 @@
     </row>
     <row r="156" spans="6:9" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="F156" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="I156" t="s">
         <v>214</v>
@@ -5922,7 +6008,7 @@
     </row>
     <row r="157" spans="6:9" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="F157" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="I157" t="s">
         <v>214</v>
@@ -5930,7 +6016,7 @@
     </row>
     <row r="158" spans="6:9" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="F158" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="I158" t="s">
         <v>214</v>
@@ -5938,7 +6024,7 @@
     </row>
     <row r="159" spans="6:9" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="F159" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="I159" t="s">
         <v>214</v>
@@ -5946,7 +6032,7 @@
     </row>
     <row r="160" spans="6:9" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="F160" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="I160" t="s">
         <v>214</v>
@@ -5954,7 +6040,7 @@
     </row>
     <row r="161" spans="4:9" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="F161" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="I161" t="s">
         <v>215</v>
@@ -5962,7 +6048,7 @@
     </row>
     <row r="162" spans="4:9" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="F162" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="I162" t="s">
         <v>215</v>
@@ -5970,7 +6056,7 @@
     </row>
     <row r="163" spans="4:9" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="F163" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="I163" t="s">
         <v>215</v>
@@ -5978,10 +6064,10 @@
     </row>
     <row r="164" spans="4:9" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="F164" t="s">
+        <v>461</v>
+      </c>
+      <c r="H164" t="s">
         <v>462</v>
-      </c>
-      <c r="H164" t="s">
-        <v>463</v>
       </c>
       <c r="I164" t="s">
         <v>215</v>
@@ -5990,13 +6076,13 @@
     <row r="165" spans="4:9" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25"/>
     <row r="166" spans="4:9" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="E166" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
     </row>
     <row r="167" spans="4:9" outlineLevel="1" x14ac:dyDescent="0.25"/>
     <row r="168" spans="4:9" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="D168" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
     </row>
     <row r="169" spans="4:9" x14ac:dyDescent="0.25">
@@ -6006,331 +6092,426 @@
     </row>
     <row r="170" spans="4:9" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="E170" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="171" spans="4:9" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="F171" t="s">
+        <v>471</v>
+      </c>
+      <c r="G171" t="s">
         <v>472</v>
-      </c>
-      <c r="G171" t="s">
-        <v>473</v>
       </c>
     </row>
     <row r="172" spans="4:9" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="F172" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
     </row>
     <row r="173" spans="4:9" outlineLevel="1" x14ac:dyDescent="0.25"/>
     <row r="174" spans="4:9" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="F174" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
     </row>
     <row r="175" spans="4:9" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="G175" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
     </row>
     <row r="176" spans="4:9" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="G176" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
     </row>
     <row r="177" spans="5:8" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="G177" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="H177" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
     </row>
     <row r="178" spans="5:8" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="G178" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="H178" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
     </row>
     <row r="179" spans="5:8" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="G179" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="H179" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
     </row>
     <row r="180" spans="5:8" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="G180" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="H180" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
     </row>
     <row r="181" spans="5:8" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="G181" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="H181" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
     </row>
     <row r="182" spans="5:8" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="G182" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="H182" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
     </row>
     <row r="183" spans="5:8" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="G183" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="H183" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
     </row>
     <row r="184" spans="5:8" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="G184" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="H184" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
     </row>
     <row r="185" spans="5:8" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="G185" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
     </row>
     <row r="186" spans="5:8" outlineLevel="1" x14ac:dyDescent="0.25"/>
     <row r="187" spans="5:8" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="E187" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
     </row>
     <row r="188" spans="5:8" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="F188" s="7" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
     </row>
     <row r="189" spans="5:8" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="F189" s="7"/>
       <c r="G189" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
     </row>
     <row r="190" spans="5:8" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="F190" s="7"/>
       <c r="G190" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
     </row>
     <row r="191" spans="5:8" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="F191" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
     </row>
     <row r="192" spans="5:8" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="F192" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
     </row>
     <row r="193" spans="5:7" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="F193" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
     </row>
     <row r="194" spans="5:7" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="F194" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
     </row>
     <row r="195" spans="5:7" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="E195" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
     </row>
     <row r="196" spans="5:7" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="F196" t="s">
+        <v>491</v>
+      </c>
+      <c r="G196" t="s">
         <v>492</v>
-      </c>
-      <c r="G196" t="s">
-        <v>493</v>
       </c>
     </row>
     <row r="197" spans="5:7" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="F197" t="s">
+        <v>489</v>
+      </c>
+      <c r="G197" t="s">
         <v>490</v>
-      </c>
-      <c r="G197" t="s">
-        <v>491</v>
       </c>
     </row>
     <row r="198" spans="5:7" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="F198" t="s">
+        <v>493</v>
+      </c>
+      <c r="G198" t="s">
         <v>494</v>
-      </c>
-      <c r="G198" t="s">
-        <v>495</v>
       </c>
     </row>
     <row r="199" spans="5:7" outlineLevel="2" x14ac:dyDescent="0.25"/>
     <row r="200" spans="5:7" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="F200" t="s">
+        <v>495</v>
+      </c>
+      <c r="G200" t="s">
         <v>496</v>
-      </c>
-      <c r="G200" t="s">
-        <v>497</v>
       </c>
     </row>
     <row r="201" spans="5:7" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="F201" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="G201" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
     </row>
     <row r="202" spans="5:7" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="F202" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="G202" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
     </row>
     <row r="203" spans="5:7" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="F203" t="s">
+        <v>501</v>
+      </c>
+      <c r="G203" t="s">
         <v>502</v>
-      </c>
-      <c r="G203" t="s">
-        <v>503</v>
       </c>
     </row>
     <row r="204" spans="5:7" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="F204" t="s">
+        <v>503</v>
+      </c>
+      <c r="G204" t="s">
         <v>504</v>
-      </c>
-      <c r="G204" t="s">
-        <v>505</v>
       </c>
     </row>
     <row r="205" spans="5:7" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="F205" t="s">
+        <v>505</v>
+      </c>
+      <c r="G205" t="s">
         <v>506</v>
-      </c>
-      <c r="G205" t="s">
-        <v>507</v>
       </c>
     </row>
     <row r="206" spans="5:7" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="F206" t="s">
+        <v>507</v>
+      </c>
+      <c r="G206" t="s">
         <v>508</v>
-      </c>
-      <c r="G206" t="s">
-        <v>509</v>
       </c>
     </row>
     <row r="207" spans="5:7" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="F207" t="s">
+        <v>509</v>
+      </c>
+      <c r="G207" t="s">
         <v>510</v>
-      </c>
-      <c r="G207" t="s">
-        <v>511</v>
       </c>
     </row>
     <row r="208" spans="5:7" outlineLevel="2" x14ac:dyDescent="0.25"/>
     <row r="209" spans="4:7" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="F209" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="G209" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
     </row>
     <row r="210" spans="4:7" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="F210" t="s">
+        <v>512</v>
+      </c>
+      <c r="G210" t="s">
         <v>513</v>
-      </c>
-      <c r="G210" t="s">
-        <v>514</v>
       </c>
     </row>
     <row r="211" spans="4:7" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="F211" t="s">
+        <v>515</v>
+      </c>
+      <c r="G211" t="s">
         <v>516</v>
-      </c>
-      <c r="G211" t="s">
-        <v>517</v>
       </c>
     </row>
     <row r="212" spans="4:7" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="F212" t="s">
+        <v>517</v>
+      </c>
+      <c r="G212" t="s">
         <v>518</v>
-      </c>
-      <c r="G212" t="s">
-        <v>519</v>
       </c>
     </row>
     <row r="213" spans="4:7" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="F213" t="s">
+        <v>519</v>
+      </c>
+      <c r="G213" t="s">
         <v>520</v>
-      </c>
-      <c r="G213" t="s">
-        <v>521</v>
       </c>
     </row>
     <row r="214" spans="4:7" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="F214" t="s">
+        <v>521</v>
+      </c>
+      <c r="G214" t="s">
         <v>522</v>
-      </c>
-      <c r="G214" t="s">
-        <v>523</v>
       </c>
     </row>
     <row r="215" spans="4:7" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="F215" t="s">
+        <v>523</v>
+      </c>
+      <c r="G215" t="s">
         <v>524</v>
-      </c>
-      <c r="G215" t="s">
-        <v>525</v>
       </c>
     </row>
     <row r="216" spans="4:7" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="E216" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
     </row>
     <row r="217" spans="4:7" outlineLevel="1" x14ac:dyDescent="0.25"/>
     <row r="218" spans="4:7" outlineLevel="1" x14ac:dyDescent="0.25"/>
     <row r="219" spans="4:7" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="D219" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
     </row>
     <row r="221" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D221" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
     </row>
     <row r="222" spans="4:7" x14ac:dyDescent="0.25">
       <c r="F222" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
     </row>
     <row r="227" spans="6:6" x14ac:dyDescent="0.25">
       <c r="F227" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
     </row>
     <row r="232" spans="6:6" x14ac:dyDescent="0.25">
       <c r="F232" t="s">
-        <v>582</v>
+        <v>581</v>
+      </c>
+    </row>
+    <row r="242" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="D242" t="s">
+        <v>583</v>
+      </c>
+    </row>
+    <row r="243" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="E243" t="s">
+        <v>586</v>
+      </c>
+    </row>
+    <row r="244" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="F244" t="s">
+        <v>588</v>
+      </c>
+    </row>
+    <row r="245" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="F245" t="s">
+        <v>587</v>
+      </c>
+    </row>
+    <row r="246" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="F246" t="s">
+        <v>599</v>
+      </c>
+    </row>
+    <row r="247" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="E247" t="s">
+        <v>593</v>
+      </c>
+    </row>
+    <row r="248" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="F248" t="s">
+        <v>584</v>
+      </c>
+    </row>
+    <row r="249" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="G249" t="s">
+        <v>590</v>
+      </c>
+    </row>
+    <row r="250" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="G250" t="s">
+        <v>591</v>
+      </c>
+    </row>
+    <row r="251" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="G251" t="s">
+        <v>589</v>
+      </c>
+    </row>
+    <row r="253" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="F253" t="s">
+        <v>585</v>
+      </c>
+    </row>
+    <row r="254" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="G254" t="s">
+        <v>592</v>
+      </c>
+    </row>
+    <row r="255" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="G255" t="s">
+        <v>594</v>
+      </c>
+    </row>
+    <row r="259" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F259" t="s">
+        <v>595</v>
+      </c>
+    </row>
+    <row r="260" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G260" t="s">
+        <v>596</v>
+      </c>
+    </row>
+    <row r="261" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G261" t="s">
+        <v>598</v>
+      </c>
+    </row>
+    <row r="262" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A262" t="s">
+        <v>597</v>
+      </c>
+    </row>
+    <row r="263" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F263" t="s">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="266" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E266" t="s">
+        <v>601</v>
       </c>
     </row>
   </sheetData>

</xml_diff>